<commit_message>
Refactor code structure for improved readability and maintainability Add industry neu, support time-range stock index universe
</commit_message>
<xml_diff>
--- a/test/eventstudy/1.春节假期.xlsx
+++ b/test/eventstudy/1.春节假期.xlsx
@@ -1,15 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27932"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6c4865365aac491c/betalens/test/eventstudy/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="1" documentId="11_403DBF94B33AF8464A3C345F18F059A054942699" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AD99D2EF-B125-4BD9-9C64-C9D26F3D10A3}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="-96" yWindow="-96" windowWidth="23232" windowHeight="12432" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
+  <extLst>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -58,15 +69,15 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
+    <numFmt numFmtId="176" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="宋体"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -74,8 +85,15 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="宋体"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="宋体"/>
+      <family val="3"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -119,20 +137,28 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="常规" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -170,7 +196,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -204,6 +230,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -238,9 +265,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -413,11 +441,14 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C11"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.1" x14ac:dyDescent="0.4"/>
+  <cols>
+    <col min="1" max="1" width="20.41796875" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -428,7 +459,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" s="2">
         <v>42407</v>
       </c>
@@ -439,7 +470,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" s="2">
         <v>42762</v>
       </c>
@@ -450,7 +481,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" s="2">
         <v>43146</v>
       </c>
@@ -461,7 +492,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" s="2">
         <v>43500</v>
       </c>
@@ -472,7 +503,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" s="2">
         <v>43854</v>
       </c>
@@ -483,7 +514,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="7" spans="1:3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7" s="2">
         <v>44238</v>
       </c>
@@ -494,7 +525,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="8" spans="1:3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A8" s="2">
         <v>44592</v>
       </c>
@@ -505,7 +536,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="1:3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A9" s="2">
         <v>44947</v>
       </c>
@@ -516,7 +547,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="1:3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A10" s="2">
         <v>45331</v>
       </c>
@@ -527,7 +558,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="11" spans="1:3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A11" s="2">
         <v>45685</v>
       </c>
@@ -539,6 +570,7 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>